<commit_message>
Sidste rettelser af modeller
</commit_message>
<xml_diff>
--- a/modeller/SOC - vælgSmiley.xlsx
+++ b/modeller/SOC - vælgSmiley.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Itzar\Desktop\Datamatiker\GitHub\HYDAC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frede\git\HYDAC\Modeller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{145C89E3-EAD6-42F9-B71F-5235ED62FA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7777B9-F9F4-44A6-B3AF-0EF0F1BB6B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="2580" windowWidth="14400" windowHeight="8170" activeTab="1" xr2:uid="{6BEF6902-C678-4111-8C9D-753D6FEAD369}"/>
+    <workbookView xWindow="1837" yWindow="1837" windowWidth="16201" windowHeight="9308" activeTab="1" xr2:uid="{6BEF6902-C678-4111-8C9D-753D6FEAD369}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -48,12 +48,6 @@
     <t>Operation:</t>
   </si>
   <si>
-    <t>SOC - System Operation Contract for vælg smiley system</t>
-  </si>
-  <si>
-    <t>UC 1: Tjek ind</t>
-  </si>
-  <si>
     <t>Postcondition 1:</t>
   </si>
   <si>
@@ -72,21 +66,9 @@
     <t>Smiley instans valgtSmiley blev oprettet</t>
   </si>
   <si>
-    <t>Medarbejder aktivMedarbejder er identificeret I systemet</t>
-  </si>
-  <si>
     <t>Output:</t>
   </si>
   <si>
-    <t>tekst</t>
-  </si>
-  <si>
-    <t>vælgSmiley(humør: grøn, rød)</t>
-  </si>
-  <si>
-    <t>valgtSmiley blev sat til humør</t>
-  </si>
-  <si>
     <t>Kvalitetskriterier</t>
   </si>
   <si>
@@ -103,6 +85,24 @@
   </si>
   <si>
     <t>Operationsnavn og parametre staves det samme som I SSDen</t>
+  </si>
+  <si>
+    <t>SOC - vælgSmiley(humør)</t>
+  </si>
+  <si>
+    <t>UC1: Tjek ind</t>
+  </si>
+  <si>
+    <t>Medarbejder aktivMedarbejder er identificeret i systemet</t>
+  </si>
+  <si>
+    <t>valgtSmiley.Farve blev sat til humør</t>
+  </si>
+  <si>
+    <t>"God dag"</t>
+  </si>
+  <si>
+    <t>vælgSmiley(humør: grøn, gul, rød)</t>
   </si>
 </sst>
 </file>
@@ -189,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -197,6 +197,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -215,7 +218,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -532,7 +535,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16B7B7D-529E-443A-9F85-DC2B808F522C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -541,107 +544,107 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E95F070-7F74-4B79-BD0A-F151C5BF3BC6}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.90625" customWidth="1"/>
-    <col min="2" max="2" width="48.1796875" customWidth="1"/>
-    <col min="4" max="4" width="81.36328125" customWidth="1"/>
+    <col min="1" max="1" width="20.9296875" customWidth="1"/>
+    <col min="2" max="2" width="48.19921875" customWidth="1"/>
+    <col min="4" max="4" width="81.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1"/>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="7"/>
       <c r="C1" s="5"/>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C2" s="6">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C3" s="6">
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="C4" s="6">
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="6">
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C6" s="6">
         <v>5</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>